<commit_message>
Deploy Tax Automation Lab v6.12.0
Updates Financial Statement to v1.2.0, TFA Client File to v1.7.0 and preserves LIPE v3.3.0 reliability fixes, together with the updated multilingual website and AI onboarding.
</commit_message>
<xml_diff>
--- a/resources/templates/TFA_Client_File_AI.xlsx
+++ b/resources/templates/TFA_Client_File_AI.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="Ra0ac9d3e96bc4a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Rd822e45ac8024565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analitica" sheetId="3" r:id="Rd878b319088f4702"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="4" r:id="R9f381871f0c9429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="Rad59bb22041146e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Re3c417ac33fc43a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analitica" sheetId="3" r:id="R038e1b71cf074c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="4" r:id="R75a5b3915171466c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -82,67 +82,27 @@
   <x:borders count="18">
     <x:border/>
     <x:border/>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:left/>
-    </x:border>
-    <x:border>
-      <x:right/>
-    </x:border>
-    <x:border>
-      <x:left/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:right/>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
-    <x:border>
-      <x:top/>
-    </x:border>
-    <x:border>
-      <x:bottom/>
-    </x:border>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
+    <x:border/>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="96">
+  <x:cellXfs count="97">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -399,6 +359,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -602,7 +563,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="92" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="85" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -616,7 +577,7 @@
         <x:v>Versione template</x:v>
       </x:c>
       <x:c r="B2" s="49" t="str">
-        <x:v>1.6.0</x:v>
+        <x:v>1.7.0</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
@@ -674,7 +635,7 @@
         <x:v>1 · Anagrafica</x:v>
       </x:c>
       <x:c r="B10" s="49" t="str">
-        <x:v>Compilare la colonna «Valore». Non modificare i codici campo. Indicare, quando possibile, fonte e stato di verifica.</x:v>
+        <x:v>Compilare la colonna «Valore». Non modificare i codici campo. Indicare, quando possibile, fonte e stato di verifica. Il periodo d’imposta deve essere espresso con quattro cifre, ad esempio 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
@@ -740,7 +701,7 @@
         <x:v>Date</x:v>
       </x:c>
       <x:c r="B19" s="49" t="str">
-        <x:v>Usare preferibilmente il formato AAAA-MM-GG.</x:v>
+        <x:v>Usare preferibilmente il formato AAAA-MM-GG. Per il periodo d’imposta usare esclusivamente un anno di quattro cifre compreso tra 2000 e 2100.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="32" customHeight="1">
@@ -748,7 +709,7 @@
         <x:v>Importi</x:v>
       </x:c>
       <x:c r="B20" s="49" t="str">
-        <x:v>Inserire numeri senza simboli di valuta; indicare la valuta nell’anagrafica o nelle note.</x:v>
+        <x:v>Inserire numeri senza simboli di valuta. Sono accettati i separatori italiani (1.234,56) e internazionali (1,234.56); indicare la valuta nell’anagrafica o nelle note.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="32" customHeight="1">
@@ -765,6 +726,52 @@
       </x:c>
       <x:c r="B22" s="53" t="str">
         <x:v>Restituire il file nello stesso formato .xlsx e accompagnarlo con un elenco separato di assunzioni, elementi mancanti e punti da validare.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="34" t="str">
+        <x:v>SALVATAGGIO E SICUREZZA DEI DATI</x:v>
+      </x:c>
+      <x:c r="B24" s="34"/>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A25" s="34" t="str">
+        <x:v>Draft locale</x:v>
+      </x:c>
+      <x:c r="B25" s="34" t="str">
+        <x:v>Durante la compilazione il browser mantiene un draft locale. Il draft non equivale al salvataggio nell’archivio del tool.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A26" s="34" t="str">
+        <x:v>Archivio del tool</x:v>
+      </x:c>
+      <x:c r="B26" s="34" t="str">
+        <x:v>Dopo l’importazione e la verifica premere «Salva nell’archivio». Il tool mostra in modo permanente se il fascicolo è archiviato o contiene modifiche non archiviate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A27" s="34" t="str">
+        <x:v>Backup completo</x:v>
+      </x:c>
+      <x:c r="B27" s="34" t="str">
+        <x:v>Esportare periodicamente l’archivio completo in JSON, soprattutto prima di cancellare i dati del browser, cambiare computer o ripristinare un backup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A28" s="34" t="str">
+        <x:v>IRL</x:v>
+      </x:c>
+      <x:c r="B28" s="34" t="str">
+        <x:v>IRL significa Information Request List: è l’elenco strutturato dei documenti e delle informazioni da richiedere e verificare.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A29" s="34" t="str">
+        <x:v>Importazione</x:v>
+      </x:c>
+      <x:c r="B29" s="34" t="str">
+        <x:v>Prima di creare un nuovo fascicolo, aggiornare quello corrente o ripristinare un backup, il tool chiede conferma quando rileva dati o modifiche non archiviate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1304,7 +1311,9 @@
       <x:c r="F30" s="35" t="str">
         <x:v>Da verificare</x:v>
       </x:c>
-      <x:c r="G30" s="66" t="str"/>
+      <x:c r="G30" s="66" t="str">
+        <x:v>Obbligatorio: anno di quattro cifre (es. 2026).</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="65" t="str">
@@ -1551,14 +1560,18 @@
       <x:c r="G44" s="70" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F2:F44">
       <x:formula1>"Confermato,Da verificare,Inferito,Non applicabile"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation operator="between" sqref="D30">
+      <x:formula1>2000</x:formula1>
+      <x:formula2>2100</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25116f15177343ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbdadf2f667e429f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5291,7 +5304,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdd61bb6e7f44a2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a9e6829880b4d20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5561,7 +5574,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cdccfa47c2d4106"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e5ceced42a5458a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Release - aggironamenti post audit 10.08.2026
</commit_message>
<xml_diff>
--- a/resources/templates/TFA_Client_File_AI.xlsx
+++ b/resources/templates/TFA_Client_File_AI.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="Rad59bb22041146e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Re3c417ac33fc43a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analitica" sheetId="3" r:id="R038e1b71cf074c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="4" r:id="R75a5b3915171466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="R8bd29252381641b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Rffc1841ae2ef478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analitica" sheetId="3" r:id="R3a4568a28f634d48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="4" r:id="R8b326a2d13db4eb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -456,9 +456,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -577,7 +577,7 @@
         <x:v>Versione template</x:v>
       </x:c>
       <x:c r="B2" s="49" t="str">
-        <x:v>1.7.0</x:v>
+        <x:v>1.7.1</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
@@ -1571,7 +1571,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbdadf2f667e429f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1321c17833e4f4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5304,7 +5304,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a9e6829880b4d20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92ebf3bfa54e4950"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5574,7 +5574,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e5ceced42a5458a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eadf2997cdd4b27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>